<commit_message>
added: programming for combinitaion mode
last switching warehouse test before heading to site
</commit_message>
<xml_diff>
--- a/Documentation/200I-25-84927_Dallas_MPR_NVX&Network.xlsx
+++ b/Documentation/200I-25-84927_Dallas_MPR_NVX&Network.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CodeStoreJBZ\Customers\B\Bain &amp; Co\Dallas TX\mpr\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11481B4C-4268-4326-8427-EEEC80148D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{654914D1-73B1-41E2-9527-138494745283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CC1CACBD-268E-4C47-A9AA-3A169F455E97}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="300">
   <si>
     <t>Analog Way Sources</t>
   </si>
@@ -914,6 +914,36 @@
   </si>
   <si>
     <t xml:space="preserve">    11  Gway    ONLINE            41794  127.000.000.001          Not Specified</t>
+  </si>
+  <si>
+    <t>DM-NVX-D30-C4426883CDC3</t>
+  </si>
+  <si>
+    <t>DM-NVX-E20-2G-C4426883A982</t>
+  </si>
+  <si>
+    <t>DM-NVX-D200-C442689425F7</t>
+  </si>
+  <si>
+    <t>DM-NVX-D200-C44268942348</t>
+  </si>
+  <si>
+    <t>DM-NVX-E20-2G-C4426883ABCC</t>
+  </si>
+  <si>
+    <t>DM-NVX-D200-C44268942E42</t>
+  </si>
+  <si>
+    <t>DM-NVX-E20-2G-C4426883AE77</t>
+  </si>
+  <si>
+    <t>DM-NVX-D200-C44268941D72</t>
+  </si>
+  <si>
+    <t>DM-NVX-D200-C442689422D9</t>
+  </si>
+  <si>
+    <t>DM-NVX-D200-C44268942F34</t>
   </si>
 </sst>
 </file>
@@ -1831,28 +1861,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P102"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" customWidth="1"/>
-    <col min="2" max="2" width="42.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.140625" customWidth="1"/>
-    <col min="6" max="6" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.42578125" customWidth="1"/>
+    <col min="1" max="1" width="9.59765625" customWidth="1"/>
+    <col min="2" max="2" width="42.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.1328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.1328125" customWidth="1"/>
+    <col min="6" max="6" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.3984375" customWidth="1"/>
     <col min="8" max="8" width="21" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" customWidth="1"/>
-    <col min="11" max="11" width="17.140625" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.140625" customWidth="1"/>
-    <col min="16" max="16" width="46.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="30.140625" customWidth="1"/>
+    <col min="9" max="9" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.3984375" customWidth="1"/>
+    <col min="11" max="11" width="17.1328125" customWidth="1"/>
+    <col min="12" max="12" width="11.59765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.3984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.59765625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.1328125" customWidth="1"/>
+    <col min="16" max="16" width="46.3984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="30.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="3" t="s">
         <v>14</v>
       </c>
@@ -1881,17 +1911,17 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="29">
         <v>21</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="29" t="s">
         <v>76</v>
       </c>
       <c r="E2" s="26" t="s">
@@ -1903,8 +1933,11 @@
       <c r="H2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I2" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1933,17 +1966,17 @@
         <v>208</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="29">
         <v>26</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="29" t="s">
         <v>76</v>
       </c>
       <c r="E4" s="26" t="s">
@@ -1956,8 +1989,11 @@
       <c r="H4" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I4" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1986,17 +2022,17 @@
         <v>208</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="29" t="s">
         <v>76</v>
       </c>
       <c r="E6" s="26" t="s">
@@ -2008,8 +2044,11 @@
       <c r="H6" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I6" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2035,7 +2074,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2044,7 +2083,7 @@
       <c r="F8" s="6"/>
       <c r="H8" s="6"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2063,7 +2102,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2082,7 +2121,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2101,7 +2140,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2109,7 +2148,7 @@
       <c r="F12" s="6"/>
       <c r="H12" s="6"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2120,7 +2159,7 @@
       <c r="F13" s="6"/>
       <c r="H13" s="6"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -2131,7 +2170,7 @@
       <c r="F14" s="6"/>
       <c r="H14" s="6"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -2142,7 +2181,7 @@
       <c r="F15" s="6"/>
       <c r="H15" s="6"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -2151,7 +2190,7 @@
       <c r="F16" s="6"/>
       <c r="H16" s="6"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -2163,7 +2202,7 @@
       <c r="F17" s="6"/>
       <c r="H17" s="6"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -2172,7 +2211,7 @@
       <c r="F18" s="6"/>
       <c r="H18" s="6"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -2181,7 +2220,7 @@
       <c r="F19" s="6"/>
       <c r="H19" s="6"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -2190,14 +2229,14 @@
       <c r="F20" s="6"/>
       <c r="H20" s="6"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A21" s="1"/>
       <c r="C21" s="5"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
       <c r="H21" s="6"/>
     </row>
-    <row r="22" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="3" t="s">
         <v>13</v>
       </c>
@@ -2226,7 +2265,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A23" s="1">
         <v>1</v>
       </c>
@@ -2252,7 +2291,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A24" s="1">
         <v>2</v>
       </c>
@@ -2278,7 +2317,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A25" s="1">
         <v>3</v>
       </c>
@@ -2304,7 +2343,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A26" s="1">
         <v>4</v>
       </c>
@@ -2330,7 +2369,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A27" s="1">
         <v>5</v>
       </c>
@@ -2356,7 +2395,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A28" s="1">
         <v>6</v>
       </c>
@@ -2382,7 +2421,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A29" s="1">
         <v>7</v>
       </c>
@@ -2411,17 +2450,17 @@
         <v>208</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A30" s="1">
         <v>8</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="D30">
+      <c r="D30" s="29">
         <v>363</v>
       </c>
       <c r="E30" s="26" t="s">
@@ -2433,18 +2472,21 @@
       <c r="H30" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I30" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A31" s="1">
         <v>9</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="30" t="s">
         <v>86</v>
       </c>
-      <c r="D31">
+      <c r="D31" s="29">
         <v>363</v>
       </c>
       <c r="E31" s="26" t="s">
@@ -2456,8 +2498,11 @@
       <c r="H31" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I31" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A32" s="1">
         <v>10</v>
       </c>
@@ -2486,17 +2531,17 @@
         <v>208</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A33" s="1">
         <v>11</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="29">
         <v>363</v>
       </c>
       <c r="E33" s="26" t="s">
@@ -2508,18 +2553,21 @@
       <c r="H33" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I33" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A34" s="1">
         <v>12</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="30" t="s">
         <v>98</v>
       </c>
-      <c r="D34">
+      <c r="D34" s="29">
         <v>363</v>
       </c>
       <c r="E34" s="26" t="s">
@@ -2531,8 +2579,11 @@
       <c r="H34" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I34" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A35" s="1">
         <v>13</v>
       </c>
@@ -2561,17 +2612,17 @@
         <v>208</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A36" s="1">
         <v>14</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="29" t="s">
         <v>94</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="D36">
+      <c r="D36" s="29">
         <v>363</v>
       </c>
       <c r="E36" s="26" t="s">
@@ -2584,18 +2635,21 @@
       <c r="H36" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I36" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A37" s="1">
         <v>15</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="29" t="s">
         <v>95</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="30" t="s">
         <v>101</v>
       </c>
-      <c r="D37">
+      <c r="D37" s="29">
         <v>363</v>
       </c>
       <c r="E37" s="26" t="s">
@@ -2608,18 +2662,21 @@
       <c r="H37" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I37" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A38" s="1">
         <v>16</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="30" t="s">
         <v>102</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="29" t="s">
         <v>118</v>
       </c>
       <c r="E38" s="26" t="s">
@@ -2631,8 +2688,11 @@
       <c r="H38" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I38" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A39" s="1">
         <v>17</v>
       </c>
@@ -2641,7 +2701,7 @@
       <c r="F39" s="6"/>
       <c r="H39" s="6"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A40" s="1">
         <v>18</v>
       </c>
@@ -2650,7 +2710,7 @@
       <c r="F40" s="6"/>
       <c r="H40" s="6"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A41" s="1">
         <v>19</v>
       </c>
@@ -2659,7 +2719,7 @@
       <c r="F41" s="6"/>
       <c r="H41" s="6"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A42" s="1">
         <v>20</v>
       </c>
@@ -2668,7 +2728,7 @@
       <c r="F42" s="6"/>
       <c r="H42" s="6"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A43" s="1">
         <v>21</v>
       </c>
@@ -2677,7 +2737,7 @@
       <c r="F43" s="6"/>
       <c r="H43" s="6"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A44" s="1">
         <v>22</v>
       </c>
@@ -2686,7 +2746,7 @@
       <c r="F44" s="6"/>
       <c r="H44" s="6"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A45" s="1">
         <v>23</v>
       </c>
@@ -2695,14 +2755,14 @@
       <c r="F45" s="6"/>
       <c r="H45" s="6"/>
     </row>
-    <row r="51" spans="7:9" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="7:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="G51" s="8"/>
       <c r="H51" s="15" t="s">
         <v>54</v>
       </c>
       <c r="I51" s="9"/>
     </row>
-    <row r="52" spans="7:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="7:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="G52" s="16" t="s">
         <v>57</v>
       </c>
@@ -2713,11 +2773,11 @@
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="7:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="7:9" x14ac:dyDescent="0.45">
       <c r="G53" s="10"/>
       <c r="I53" s="11"/>
     </row>
-    <row r="54" spans="7:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="7:9" x14ac:dyDescent="0.45">
       <c r="G54" s="10" t="s">
         <v>49</v>
       </c>
@@ -2726,64 +2786,64 @@
       </c>
       <c r="I54" s="11"/>
     </row>
-    <row r="55" spans="7:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="7:9" x14ac:dyDescent="0.45">
       <c r="G55" s="10"/>
       <c r="H55" t="s">
         <v>51</v>
       </c>
       <c r="I55" s="11"/>
     </row>
-    <row r="56" spans="7:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="7:9" x14ac:dyDescent="0.45">
       <c r="G56" s="10"/>
       <c r="H56" t="s">
         <v>52</v>
       </c>
       <c r="I56" s="11"/>
     </row>
-    <row r="57" spans="7:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="7:9" x14ac:dyDescent="0.45">
       <c r="G57" s="10"/>
       <c r="H57" t="s">
         <v>53</v>
       </c>
       <c r="I57" s="11"/>
     </row>
-    <row r="58" spans="7:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="7:9" x14ac:dyDescent="0.45">
       <c r="G58" s="10"/>
       <c r="I58" s="11"/>
     </row>
-    <row r="59" spans="7:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="7:9" x14ac:dyDescent="0.45">
       <c r="G59" s="12" t="s">
         <v>120</v>
       </c>
       <c r="H59" s="13"/>
       <c r="I59" s="14"/>
     </row>
-    <row r="81" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="15:16" x14ac:dyDescent="0.45">
       <c r="P81" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O82">
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O83">
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O84">
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O85">
         <v>4</v>
       </c>
     </row>
-    <row r="86" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O86">
         <v>5</v>
       </c>
@@ -2791,7 +2851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O87">
         <v>6</v>
       </c>
@@ -2799,7 +2859,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O88">
         <v>7</v>
       </c>
@@ -2807,7 +2867,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="89" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O89">
         <v>8</v>
       </c>
@@ -2815,7 +2875,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O90">
         <v>9</v>
       </c>
@@ -2823,7 +2883,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="91" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O91">
         <v>10</v>
       </c>
@@ -2831,7 +2891,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="92" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O92">
         <v>11</v>
       </c>
@@ -2839,7 +2899,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="93" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O93">
         <v>12</v>
       </c>
@@ -2847,7 +2907,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O94">
         <v>13</v>
       </c>
@@ -2855,12 +2915,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="100" spans="15:16" x14ac:dyDescent="0.45">
       <c r="P100" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="101" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="101" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O101">
         <v>1</v>
       </c>
@@ -2868,7 +2928,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="15:16" x14ac:dyDescent="0.25">
+    <row r="102" spans="15:16" x14ac:dyDescent="0.45">
       <c r="O102">
         <v>2</v>
       </c>
@@ -2893,148 +2953,148 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4CA42E4-99C2-465A-8663-77A4827CB989}">
   <dimension ref="A1:A30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A1" s="23" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A2" s="23"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A3" s="23" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A4" s="23" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A5" s="23" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A6" s="23" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A7" s="23" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A8" s="23" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A9" s="23" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A10" s="23" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A11" s="23" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A12" s="23"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A13" s="23" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A14" s="23"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A15" s="23" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A16" s="23" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A17" s="23" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A18" s="23" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A19" s="23" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A20" s="23" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A21" s="23" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A22" s="23" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A23" s="23" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A24" s="23" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A25" s="23" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A26" s="23" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A27" s="23" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A28" s="23" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A29" s="23" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A30" s="23" t="s">
         <v>168</v>
       </c>
@@ -3047,18 +3107,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFEC39CD-2593-4516-8802-B56C6A059957}">
   <dimension ref="A1:I65"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.73046875" customWidth="1"/>
+    <col min="4" max="4" width="10.1328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.73046875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="7" customFormat="1" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="7" customFormat="1" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A1" s="7" t="s">
         <v>37</v>
       </c>
@@ -3084,7 +3144,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>36</v>
       </c>
@@ -3106,7 +3166,7 @@
       <c r="H2" s="21"/>
       <c r="I2" s="21"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>56</v>
       </c>
@@ -3123,7 +3183,7 @@
       <c r="H3" s="21"/>
       <c r="I3" s="21"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>56</v>
       </c>
@@ -3140,7 +3200,7 @@
       <c r="H4" s="21"/>
       <c r="I4" s="21"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>56</v>
       </c>
@@ -3157,7 +3217,7 @@
       <c r="H5" s="21"/>
       <c r="I5" s="21"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D6" s="21"/>
       <c r="E6" s="21"/>
       <c r="F6" s="21"/>
@@ -3165,7 +3225,7 @@
       <c r="H6" s="21"/>
       <c r="I6" s="21"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>60</v>
       </c>
@@ -3182,7 +3242,7 @@
       <c r="H7" s="21"/>
       <c r="I7" s="21"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>60</v>
       </c>
@@ -3199,7 +3259,7 @@
       <c r="H8" s="21"/>
       <c r="I8" s="21"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>60</v>
       </c>
@@ -3216,7 +3276,7 @@
       <c r="H9" s="21"/>
       <c r="I9" s="21"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D10" s="21"/>
       <c r="E10" s="21"/>
       <c r="F10" s="21"/>
@@ -3224,7 +3284,7 @@
       <c r="H10" s="21"/>
       <c r="I10" s="21"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="20" t="s">
         <v>145</v>
       </c>
@@ -3237,7 +3297,7 @@
       </c>
       <c r="I11" s="21"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="20" t="s">
         <v>148</v>
       </c>
@@ -3250,7 +3310,7 @@
       </c>
       <c r="I12" s="21"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D13" s="21"/>
       <c r="E13" s="21"/>
       <c r="F13" s="21"/>
@@ -3258,7 +3318,7 @@
       <c r="H13" s="21"/>
       <c r="I13" s="21"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>104</v>
       </c>
@@ -3275,7 +3335,7 @@
       <c r="H14" s="21"/>
       <c r="I14" s="21"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A15" s="19" t="s">
         <v>105</v>
       </c>
@@ -3292,7 +3352,7 @@
       <c r="H15" s="21"/>
       <c r="I15" s="21"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>106</v>
       </c>
@@ -3309,7 +3369,7 @@
       <c r="H16" s="21"/>
       <c r="I16" s="21"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A17" s="19" t="s">
         <v>107</v>
       </c>
@@ -3326,7 +3386,7 @@
       <c r="H17" s="21"/>
       <c r="I17" s="21"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>108</v>
       </c>
@@ -3343,7 +3403,7 @@
       <c r="H18" s="21"/>
       <c r="I18" s="21"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A19" s="19" t="s">
         <v>109</v>
       </c>
@@ -3354,7 +3414,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>110</v>
       </c>
@@ -3365,30 +3425,30 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
       <c r="B21" s="5"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A28" s="34" t="s">
         <v>289</v>
       </c>
@@ -3396,7 +3456,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A29" s="34" t="s">
         <v>218</v>
       </c>
@@ -3404,7 +3464,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A30" s="34" t="s">
         <v>219</v>
       </c>
@@ -3412,7 +3472,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>220</v>
       </c>
@@ -3420,7 +3480,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>221</v>
       </c>
@@ -3428,7 +3488,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>222</v>
       </c>
@@ -3436,7 +3496,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>223</v>
       </c>
@@ -3444,7 +3504,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A35" s="34" t="s">
         <v>224</v>
       </c>
@@ -3452,7 +3512,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A36" s="34" t="s">
         <v>225</v>
       </c>
@@ -3460,7 +3520,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A37" s="34" t="s">
         <v>226</v>
       </c>
@@ -3468,7 +3528,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>227</v>
       </c>
@@ -3476,7 +3536,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A39" s="34" t="s">
         <v>228</v>
       </c>
@@ -3484,7 +3544,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40" s="34" t="s">
         <v>229</v>
       </c>
@@ -3492,7 +3552,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41" s="34" t="s">
         <v>230</v>
       </c>
@@ -3500,7 +3560,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>231</v>
       </c>
@@ -3508,7 +3568,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A43" s="34" t="s">
         <v>232</v>
       </c>
@@ -3516,7 +3576,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A44" s="34" t="s">
         <v>233</v>
       </c>
@@ -3524,7 +3584,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A45" s="34" t="s">
         <v>234</v>
       </c>
@@ -3532,7 +3592,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A46" s="34" t="s">
         <v>235</v>
       </c>
@@ -3540,7 +3600,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>236</v>
       </c>
@@ -3548,7 +3608,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>237</v>
       </c>
@@ -3556,7 +3616,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A49" s="34" t="s">
         <v>238</v>
       </c>
@@ -3564,7 +3624,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>239</v>
       </c>
@@ -3572,7 +3632,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>240</v>
       </c>
@@ -3580,7 +3640,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A52" s="34" t="s">
         <v>241</v>
       </c>
@@ -3588,7 +3648,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
         <v>242</v>
       </c>
@@ -3601,7 +3661,7 @@
       </c>
       <c r="I53" s="9"/>
     </row>
-    <row r="54" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A54" t="s">
         <v>243</v>
       </c>
@@ -3618,7 +3678,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>244</v>
       </c>
@@ -3628,7 +3688,7 @@
       <c r="G55" s="10"/>
       <c r="I55" s="11"/>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>245</v>
       </c>
@@ -3643,7 +3703,7 @@
       </c>
       <c r="I56" s="11"/>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>246</v>
       </c>
@@ -3656,7 +3716,7 @@
       </c>
       <c r="I57" s="11"/>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>247</v>
       </c>
@@ -3669,7 +3729,7 @@
       </c>
       <c r="I58" s="11"/>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>248</v>
       </c>
@@ -3682,7 +3742,7 @@
       </c>
       <c r="I59" s="11"/>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>249</v>
       </c>
@@ -3692,7 +3752,7 @@
       <c r="G60" s="10"/>
       <c r="I60" s="11"/>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>250</v>
       </c>
@@ -3705,7 +3765,7 @@
       <c r="H61" s="13"/>
       <c r="I61" s="14"/>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>251</v>
       </c>
@@ -3713,7 +3773,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>252</v>
       </c>
@@ -3721,7 +3781,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>253</v>
       </c>
@@ -3729,7 +3789,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>288</v>
       </c>
@@ -3746,20 +3806,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7AAB32A-44CF-47EA-A671-55D47AC57CDE}">
   <dimension ref="A1:H50"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.73046875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.1328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="7" customFormat="1" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="7" customFormat="1" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A1" s="7" t="s">
         <v>44</v>
       </c>
@@ -3785,7 +3845,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="7" customFormat="1" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" s="7" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A2" s="7" t="s">
         <v>176</v>
       </c>
@@ -3802,7 +3862,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>181</v>
       </c>
@@ -3819,7 +3879,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>181</v>
       </c>
@@ -3836,7 +3896,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>181</v>
       </c>
@@ -3853,79 +3913,79 @@
         <v>183</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A25" s="18"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A26" s="18"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A27" s="18"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A28" s="18"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A29" s="18"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A30" s="18"/>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A31" s="18"/>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A32" s="18"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A33" s="18"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A34" s="18"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A35" s="18"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A36" s="18"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A37" s="18"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A38" s="18"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A39" s="18"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A40" s="18"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A41" s="18"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A42" s="18"/>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A43" s="18"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A44" s="18"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A45" s="18"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A46" s="18"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A47" s="18"/>
     </row>
-    <row r="49" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="6:6" x14ac:dyDescent="0.45">
       <c r="F49" s="18"/>
     </row>
-    <row r="50" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="6:6" x14ac:dyDescent="0.45">
       <c r="F50" s="18"/>
     </row>
   </sheetData>
@@ -3935,6 +3995,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FA3C1439872DC64B884A7795FD0E820C" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe0c567e1faf0c6f0064e03bad84412f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="a86625aa-26de-4d9c-bf0d-dbf15aee1a6c" xmlns:ns4="95262377-04f9-4475-9458-b3c59b0f0756" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="38a8e08ffe20c54ac34c5da0713fcd62" ns3:_="" ns4:_="">
     <xsd:import namespace="a86625aa-26de-4d9c-bf0d-dbf15aee1a6c"/>
@@ -4177,22 +4252,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29BC7EA8-9756-495D-861B-8F24EC6A2CD3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="95262377-04f9-4475-9458-b3c59b0f0756"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a86625aa-26de-4d9c-bf0d-dbf15aee1a6c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6EE3758A-99D0-4D35-B054-6BD8D048F617}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D03DF91B-FBD6-4152-B63F-184DF746E19F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4209,29 +4294,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6EE3758A-99D0-4D35-B054-6BD8D048F617}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29BC7EA8-9756-495D-861B-8F24EC6A2CD3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="95262377-04f9-4475-9458-b3c59b0f0756"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a86625aa-26de-4d9c-bf0d-dbf15aee1a6c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>